<commit_message>
Revisões: revisão de humor restrita a artigos completos em periódicos (34 estudos)
Saem o preprint de Bugten et al. (2026), o trabalho em anais de Nugraha et al.
(2020) e o resumo de congresso de Ratz-Sulyok et al. (2026); PRISMA, tabelas,
texto, apêndices, versões ABNT, MDPI e do orientador e planilhas regravados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YXxWHB8jopLfGkYhcAQesG
</commit_message>
<xml_diff>
--- a/data/revisoes/handebol/atualizacao_humor_2026-10/artigos_perfil_humor_handebol.xlsx
+++ b/data/revisoes/handebol/atualizacao_humor_2026-10/artigos_perfil_humor_handebol.xlsx
@@ -2561,7 +2561,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>(RATZ-SULYOK et al., 2026b)</t>
+          <t>(RATZ-SULYOK et al., 2026)</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>(RATZ-SULYOK et al., 2026b)</t>
+          <t>(RATZ-SULYOK et al., 2026)</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -15824,87 +15824,79 @@
       </c>
     </row>
     <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Incluído na revisão sistemática</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Excluído da revisão: não é artigo completo em periódico</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Preprint</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Preprint sem revisão por pares (Research Square).</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Youth Players Basic Need Satisfaction, Enjoyment and Pleasure within daily team sport training sessions, and the relationships with Physical Load Engagement: An intensive within-person longitudinal study</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>BUGTEN, Jesper Barth; HAUGEN, Tommy; SPENCER, Matt; IVARSSON, Andreas; BYRKJEDAL, Per Thomas; STENLING, Andreas; SOLSTAD, Bård Erlend</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Research Square (preprint)</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Bugten JB, Haugen T, Spencer M, Ivarsson A, Byrkjedal PT, Stenling A, Solstad BE.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>10.21203/rs.3.rs-8338987/v1</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>https://www.researchsquare.com/article/rs-8338987/latest.pdf</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>acceptedVersion</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Feeling Scale (Hardy; Rejeski, 1989), item único de -5 a +5, versão norueguesa adaptada</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Feeling Scale (Hardy e Rejeski, 1989)</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>não</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>(BUGTEN et al., 2026)</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>revisão (leitura integral)</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>N6</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>texto completo</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>Youth team-sport training sessions provide repeated opportunities for skill development, yet little is known about how athletes’ momentary psychological experiences relate to their physical engagement in training. Fifty adolescent female handball players (M = 14.57, SD = 1.03) completed brief questionnaires before and after 11–12 consecutive team training sessions, while physical load (PlayerLoad™) and high-intensity events (&gt; 1.5 m/s²) were recorded via inertial measurement units during training. Bayesian within-person analysis revealed temporal stability in basic need satisfaction, sport enjoyment, and feelings of pleasure before and after training. Before and after training, basic needs satisfaction was associated with sport enjoyment and pleasure. Pleasure before training was associated with physical load during training, which was further associated with pleasure after training. This highlights that youth athletes’ basic need satisfaction and affective experiences are intertwined with their physical engagement in training, underscoring the importance of creating need-supportive training environments that foster both positive affect and meaningful behavioral involvement for athlete development in youth sport.</t>
+      <c r="M3" s="4" t="inlineStr"/>
+      <c r="N3" s="4" t="inlineStr"/>
+      <c r="O3" s="4" t="inlineStr"/>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>busca 1 (PubMed, Europe PMC, Crossref)</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>N162</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr"/>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>&lt;title&gt;Abstract&lt;/title&gt;  &lt;p&gt;Youth team-sport training sessions provide repeated opportunities for skill development, yet little is known about how athletes’ momentary psychological experiences relate to their physical engagement in training. Fifty adolescent female handball players (M = 14.57, SD = 1.03) completed brief questionnaires before and after 11–12 consecutive team training sessions, while physical load (PlayerLoad™) and high-intensity events (&gt; 1.5 m/s²) were recorded via inertial measurement units during training. Bayesian within-person analysis revealed temporal stability in basic need satisfaction, sport enjoyment, and feelings of pleasure before and after training. Before and after training, basic needs satisfaction was associated with sport enjoyment and pleasure. Pleasure before training was associated with physical load during training, which was further associated with pleasure after training. This highlights that youth athletes’ basic need satisfaction and affective experiences are intertwined with their physical engagement in training, underscoring the importance of creating need-supportive training environments that foster both positive affect and meaningful behavioral involvement for athlete development in youth sport.&lt;/p&gt;</t>
         </is>
       </c>
     </row>
@@ -16037,91 +16029,86 @@
       </c>
     </row>
     <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Incluído na revisão sistemática</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Excluído da revisão: não é artigo completo em periódico</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Resumo de congresso</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Resumo de congresso (suplemento) da amostra de Ratz-Sulyok et al. (2026), estudo H34.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Stress and sex hormone changes of young elite handball players in relation to their mood profiles</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>RATZ-SULYOK, Fanny Zselyke; JANG-KAPUY, Csilla; BAKONYI, Peter; BERES, Bettina; DOBRONYI, Tamas; SIMON, Gergo; ZSAKAI, Annamaria; SZABO, Tamas</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Ratz-Sulyok; Jang-Kapuy; Bakonyi; Beres</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Anthropologiai Közlemények</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>10.20330/anthropkozl.2026.67s.108</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>https://ojs.mtak.hu/index.php/anthropkozl/article/download/24429/20220</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>publishedVersion</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>POMS-65</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>POMS</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>não relatado</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>584</v>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>(RATZ-SULYOK et al., 2026a)</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>revisão (leitura integral)</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>N9</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>resumo</t>
-        </is>
-      </c>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Background: Excessive training-induced stress in athletes is theorised to cause maladaptation in athletes, when there is an imbalance in training and recovery, which can later lead to overtraining syndrome (OTS). OTS detection is prominently based on the change of testosterone and cortisol levels due to maximal exertion, alongside mood profiling. Objective: To study the relationship between mood profile, stress state, endocrine status and response to physical exertion in youth handball players. The analysis is part of a large study to develop a new screening method for overtraining status in athletes. Subjects and methods: 584 elite Hungarian handball players (14–35 ys) were examined in the Sport Sciences and Diagnostic Research Centre of the Hungarian Handball Federation between 2023 and 2025. Saliva samples were collected in resting state and after vital maximum exertion to measure the concentration of testosterone and cortisol, and 17-β-oestradiol hormone levels. Hormone levels were estimated by ELISA method. Subjective stress state of the athletes was surveyed via Profile of Mood States questionnaire. Results: The athlete references of resting levels of sex hormones, as well as the change in the ratio of sex hormone and cortisol hormone levels were constructed for athletes. Sex hormone levels showed deviations from the non-athlete references in both sexes: the resting testosterone level of male athletes was higher, while 17-β-oestradiol level of female athletes was lower </t>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>busca 1 (PubMed, Europe PMC, Crossref)</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>N163</t>
+        </is>
+      </c>
+      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>Background: Excessive training-induced stress in athletes is theorised to cause maladaptation in athletes, when there is an imbalance in training and recovery, which can later lead to overtraining syndrome (OTS). OTS detection is prominently based on the change of testosterone and cortisol levels due to maximal exertion, alongside mood profiling.
+Objective: To study the relationship between mood profile, stress state, endocrine status and response to physical exertion in youth handball players. The analysis is part of a large study to develop a new screening method for overtraining status in athletes.  
+Subjects and methods: 584 elite Hungarian handball players (14–35 ys) were examined in the Sport Sciences and Diagnostic Research Centre of the Hungarian Handball Federation between 2023 and 2025. Saliva samples were collected in resting state and after vital maximum exertion to measure the concentration of testosterone and cortisol, and 17-β-oestradiol hormone levels. Hormone levels were estimated by ELISA method. Subjective stress state of the athletes was surveyed via Profile of Mood States questionnaire.
+Results: The athlete references of resting levels of sex hormones, as well as the change in the ratio of sex hormone and cortisol hormone levels were constructed for athletes. Sex hormone levels showed deviations from the non-athlete references in both sexes: the resting testosterone level of male athletes was higher, while 17-β-oestradiol level of female athletes was l</t>
         </is>
       </c>
     </row>
@@ -17724,87 +17711,83 @@
       </c>
     </row>
     <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Incluído na revisão sistemática</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Excluído da revisão: não é artigo completo em periódico</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Trabalho em anais de congresso</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Trabalho completo em anais de congresso (Atlantis Press).</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Mood States and Game Performance in Invasion Game Activities: A Correlation Study Among Elementary School Students</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>NUGRAHA, Eka; WIBOWO, Ricky; FIRMANSYAH, Helmy</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>E. Nugraha; R. Wibowo; H. Firmansyah</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>Proceedings of the 4th International Conference on Sport Science, Health, and Physical Education (ICSSHPE 2019)</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>10.2991/ahsr.k.200214.027</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>https://www.atlantis-press.com/article/125934764.pdf</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>publishedVersion</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Brief Mood Introspection Scale (BMIS), 16 itens, escala Likert de 4 pontos (adaptada)</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Brief Mood Introspection Scale (BMIS)</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>não</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>(NUGRAHA; WIBOWO; FIRMANSYAH, 2020)</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>revisão (leitura integral)</t>
-        </is>
-      </c>
-      <c r="Q30" s="2" t="inlineStr">
+      <c r="M30" s="4" t="inlineStr"/>
+      <c r="N30" s="4" t="inlineStr"/>
+      <c r="O30" s="4" t="inlineStr"/>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>busca 2 (Semantic Scholar, Dialnet)</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr">
         <is>
           <t>U107</t>
         </is>
       </c>
-      <c r="R30" s="2" t="inlineStr">
-        <is>
-          <t>texto completo</t>
-        </is>
-      </c>
-      <c r="S30" s="2" t="inlineStr">
-        <is>
-          <t>Children play games for the same reason. They play because playing is fun. Interest to games may have meaningful psychological benefits for children. The purpose of this study was to examine the association between short-term psychological effects, especially moods states, and games performance in invasion game activities setting at elementary students. Correlational approach was used to analyse the results of this study. Third grade elementary school students were enrolled in this study. Forty elementary students were assigned to invasion games in 8 minute game, which was divided into two minute halves. The game taught used invasion games was handball, which fields size and rules were modified. Pleasant and unpleasant moods using Brief Mood Introspection Scale (BMIS) were assessed before experimental conditions. BMIS with 8 sub-scales pleasant mood states (active, calm, caring, content, happy, lively, loving, and peppy) and unpleasant mood states (drowsy, fed up, gloomy, grouchy, jittery, nervous, sad, and tired) are rated on a 4-point Likert scale ranging from 1 (definitely do not feel) to 4 (definitely feel). It was found that pleasant moods states correlated with games performance and games involvement of the student in games activities. This study suggests physical educators to setting motivated climate to increase moods states in order to engage children in physical activities.</t>
+      <c r="R30" s="4" t="inlineStr"/>
+      <c r="S30" s="4" t="inlineStr">
+        <is>
+          <t>Children play games for the same reason. They play because playing is fun. Interest to games may have meaningful psychological benefits for children. The purpose of this study was to examine the association between short-term psychological effects, especially moods states, and games performance in invasion game activities setting at elementary students. Correlational approach was used to analyse the results of this study. Third grade elementary school students were enrolled in this study. Forty elementary students were assigned to invasion games in 8 minute game, which was divided into two minute halves. The game taught used invasion games was handball, which fields size and rules were modified. Pleasant and unpleasant moods using Brief Mood Introspection Scale (BMIS) were assessed before experimental conditions. BMIS with 8 subscales pleasant mood states (active, calm, caring, content, happy, lively, loving, and peppy) and unpleasant mood states (drowsy, fed up, gloomy, grouchy, jittery, nervous, sad, and tired) are rated on a 4-point Likert scale ranging from 1 (definitely do not feel) to 4 (definitely feel). It was found that pleasant moods states correlated with games performance and games involvement of the student in games activities. This study suggests physical educators to setting motivated climate to increase moods states in order to engage children in physical activities.</t>
         </is>
       </c>
     </row>

</xml_diff>